<commit_message>
251225 ver2_0 完成☆　最終版として保存 --------------------------------------
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel/Entity_ContestStartListDataBase.xlsx
+++ b/Assets/Resources/Excel/Entity_ContestStartListDataBase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aritashogo\Documents\Unity\Okashi_Atlier2\Assets\Resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1D9786-F2F8-40FB-B27C-EDCF6E666EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03DE650-BECC-4755-93E0-75F06A5AFD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3225" yWindow="1380" windowWidth="25005" windowHeight="14370" xr2:uid="{1DCE2773-8A3B-4011-B3F4-E2EABC03DB8B}"/>
+    <workbookView xWindow="2340" yWindow="1830" windowWidth="25005" windowHeight="14370" xr2:uid="{1DCE2773-8A3B-4011-B3F4-E2EABC03DB8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Or_Contest_001" sheetId="1" r:id="rId1"/>
@@ -636,48 +636,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>◆秋の伝統的なお菓子コンクール◆
-テーマ：自由課題
-秋エリアの伝統的で由緒あるコンクールです。食べた人を幸せにするお菓子をお待ちしております。</t>
-    <rPh sb="1" eb="2">
-      <t>アキ</t>
-    </rPh>
-    <rPh sb="3" eb="6">
-      <t>デントウテキ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="26" eb="27">
-      <t>アキ</t>
-    </rPh>
-    <rPh sb="31" eb="33">
-      <t>デントウ</t>
-    </rPh>
-    <rPh sb="33" eb="34">
-      <t>テキ</t>
-    </rPh>
-    <rPh sb="35" eb="37">
-      <t>ユイショ</t>
-    </rPh>
-    <rPh sb="47" eb="48">
-      <t>タ</t>
-    </rPh>
-    <rPh sb="50" eb="51">
-      <t>ヒト</t>
-    </rPh>
-    <rPh sb="52" eb="53">
-      <t>シアワ</t>
-    </rPh>
-    <rPh sb="58" eb="60">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="62" eb="63">
-      <t>マ</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>マジカル・パティスリー・アワード</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -1174,51 +1132,6 @@
     </rPh>
     <rPh sb="47" eb="48">
       <t>ミ</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>◆お子様向けのお菓子限定◆
-お子様が喜ぶ色々なお菓子を募集しています！
-かわいいや不思議なお菓子など.. ぜひ応募お待ちしてます！</t>
-    <rPh sb="2" eb="4">
-      <t>コサマ</t>
-    </rPh>
-    <rPh sb="4" eb="5">
-      <t>ム</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t>ゲンテイ</t>
-    </rPh>
-    <rPh sb="15" eb="17">
-      <t>コサマ</t>
-    </rPh>
-    <rPh sb="18" eb="19">
-      <t>ヨロコ</t>
-    </rPh>
-    <rPh sb="20" eb="22">
-      <t>イロイロ</t>
-    </rPh>
-    <rPh sb="24" eb="26">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="27" eb="29">
-      <t>ボシュウ</t>
-    </rPh>
-    <rPh sb="41" eb="44">
-      <t>フシギ</t>
-    </rPh>
-    <rPh sb="46" eb="48">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="55" eb="57">
-      <t>オウボ</t>
-    </rPh>
-    <rPh sb="58" eb="59">
-      <t>マ</t>
     </rPh>
     <phoneticPr fontId="2"/>
   </si>
@@ -1964,46 +1877,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>◆夏エリア最大のお菓子エキシビジョン◆
-テーマ：自由課題
-ソーダアイランドで行われるお菓子の一大イベント！
-自慢のお菓子で来客者を喜ばせよう！！</t>
-    <rPh sb="1" eb="2">
-      <t>ナツ</t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t>サイダイ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="24" eb="28">
-      <t>ジユウカダイ</t>
-    </rPh>
-    <rPh sb="38" eb="39">
-      <t>オコナ</t>
-    </rPh>
-    <rPh sb="43" eb="45">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="46" eb="48">
-      <t>イチダイ</t>
-    </rPh>
-    <rPh sb="54" eb="56">
-      <t>ジマン</t>
-    </rPh>
-    <rPh sb="58" eb="60">
-      <t>カシ</t>
-    </rPh>
-    <rPh sb="61" eb="64">
-      <t>ライキャクシャ</t>
-    </rPh>
-    <rPh sb="65" eb="66">
-      <t>ヨロコ</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>◆パティシエアカデミーの登竜門◆
 テーマ：焼き菓子と自由課題
 来たれ！パティシエのたまごたちよ！
@@ -2345,6 +2218,129 @@
   </si>
   <si>
     <t>h05</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>◆夏エリア最大のお菓子エキシビジョン◆
+テーマ：焼き菓子・自由課題ほか
+ソーダアイランドで行われるお菓子の一大イベント！自慢のお菓子でお客さんを喜ばせよう！！</t>
+    <rPh sb="1" eb="2">
+      <t>ナツ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>サイダイ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="24" eb="25">
+      <t>ヤ</t>
+    </rPh>
+    <rPh sb="26" eb="28">
+      <t>ガシ</t>
+    </rPh>
+    <rPh sb="29" eb="33">
+      <t>ジユウカダイ</t>
+    </rPh>
+    <rPh sb="45" eb="46">
+      <t>オコナ</t>
+    </rPh>
+    <rPh sb="50" eb="52">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="53" eb="55">
+      <t>イチダイ</t>
+    </rPh>
+    <rPh sb="60" eb="62">
+      <t>ジマン</t>
+    </rPh>
+    <rPh sb="64" eb="66">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="68" eb="69">
+      <t>キャク</t>
+    </rPh>
+    <rPh sb="72" eb="73">
+      <t>ヨロコ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>◆秋の伝統的なお菓子コンクール◆
+テーマ：自由課題
+秋エリアの伝統的で由緒あるコンクールです。自信作をお待ちしております。</t>
+    <rPh sb="1" eb="2">
+      <t>アキ</t>
+    </rPh>
+    <rPh sb="3" eb="6">
+      <t>デントウテキ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="26" eb="27">
+      <t>アキ</t>
+    </rPh>
+    <rPh sb="31" eb="33">
+      <t>デントウ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="35" eb="37">
+      <t>ユイショ</t>
+    </rPh>
+    <rPh sb="47" eb="50">
+      <t>ジシンサク</t>
+    </rPh>
+    <rPh sb="52" eb="53">
+      <t>マ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>◆お子様向けのお菓子限定◆
+お子様が喜ぶ色々なお菓子を募集しています！
+キャンディや不思議なお菓子など.. ぜひ応募お待ちしてます！</t>
+    <rPh sb="2" eb="4">
+      <t>コサマ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ム</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ゲンテイ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>コサマ</t>
+    </rPh>
+    <rPh sb="18" eb="19">
+      <t>ヨロコ</t>
+    </rPh>
+    <rPh sb="20" eb="22">
+      <t>イロイロ</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="27" eb="29">
+      <t>ボシュウ</t>
+    </rPh>
+    <rPh sb="42" eb="45">
+      <t>フシギ</t>
+    </rPh>
+    <rPh sb="47" eb="49">
+      <t>カシ</t>
+    </rPh>
+    <rPh sb="56" eb="58">
+      <t>オウボ</t>
+    </rPh>
+    <rPh sb="59" eb="60">
+      <t>マ</t>
+    </rPh>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2787,7 +2783,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -2847,7 +2843,7 @@
         <v>98</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>19</v>
@@ -2961,10 +2957,10 @@
         <v>9</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -3048,10 +3044,10 @@
         <v>87</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -3099,10 +3095,10 @@
         <v>0</v>
       </c>
       <c r="W4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="X4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="Y4" t="s">
         <v>101</v>
@@ -3135,10 +3131,10 @@
         <v>73</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -3225,7 +3221,7 @@
         <v>83</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -3240,7 +3236,7 @@
         <v>31</v>
       </c>
       <c r="L6">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="M6">
         <v>3</v>
@@ -3273,7 +3269,7 @@
         <v>0</v>
       </c>
       <c r="W6" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="X6" t="s">
         <v>99</v>
@@ -3309,10 +3305,10 @@
         <v>84</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -3336,7 +3332,7 @@
         <v>2</v>
       </c>
       <c r="O7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -3360,13 +3356,13 @@
         <v>0</v>
       </c>
       <c r="W7" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="X7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="Y7" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z7">
         <v>3</v>
@@ -3396,10 +3392,10 @@
         <v>70</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -3483,10 +3479,10 @@
         <v>78</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -3570,10 +3566,10 @@
         <v>85</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -3588,7 +3584,7 @@
         <v>31</v>
       </c>
       <c r="L10">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="M10">
         <v>5</v>
@@ -3621,13 +3617,13 @@
         <v>0</v>
       </c>
       <c r="W10" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="X10" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="Y10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z10">
         <v>3</v>
@@ -3651,16 +3647,16 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -3708,13 +3704,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="X11" t="s">
         <v>99</v>
       </c>
       <c r="Y11" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z11">
         <v>3</v>
@@ -3744,10 +3740,10 @@
         <v>71</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -3831,10 +3827,10 @@
         <v>29</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -3882,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="W13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="X13" t="s">
         <v>99</v>
@@ -3941,7 +3937,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -4001,7 +3997,7 @@
         <v>98</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>19</v>
@@ -4028,10 +4024,10 @@
         <v>65</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -4079,10 +4075,10 @@
         <v>0</v>
       </c>
       <c r="W2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y2" t="s">
         <v>101</v>
@@ -4109,16 +4105,16 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -4142,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P3">
         <v>1</v>
@@ -4166,13 +4162,13 @@
         <v>0</v>
       </c>
       <c r="W3" t="s">
+        <v>130</v>
+      </c>
+      <c r="X3" t="s">
         <v>131</v>
       </c>
-      <c r="X3" t="s">
-        <v>132</v>
-      </c>
       <c r="Y3" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="Z3">
         <v>2</v>
@@ -4202,10 +4198,10 @@
         <v>91</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -4253,10 +4249,10 @@
         <v>0</v>
       </c>
       <c r="W4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y4" t="s">
         <v>101</v>
@@ -4289,10 +4285,10 @@
         <v>89</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -4319,7 +4315,7 @@
         <v>2</v>
       </c>
       <c r="P5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>99</v>
@@ -4340,10 +4336,10 @@
         <v>0</v>
       </c>
       <c r="W5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y5" t="s">
         <v>101</v>
@@ -4370,16 +4366,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -4403,7 +4399,7 @@
         <v>10</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -4427,10 +4423,10 @@
         <v>0</v>
       </c>
       <c r="W6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y6" t="s">
         <v>101</v>
@@ -4463,10 +4459,10 @@
         <v>66</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -4514,10 +4510,10 @@
         <v>0</v>
       </c>
       <c r="W7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y7" t="s">
         <v>101</v>
@@ -4553,7 +4549,7 @@
         <v>67</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -4601,13 +4597,13 @@
         <v>0</v>
       </c>
       <c r="W8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="X8" t="s">
         <v>99</v>
       </c>
       <c r="Y8" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z8">
         <v>3</v>
@@ -4640,7 +4636,7 @@
         <v>90</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -4655,7 +4651,7 @@
         <v>31</v>
       </c>
       <c r="L9">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="M9">
         <v>12</v>
@@ -4664,7 +4660,7 @@
         <v>20</v>
       </c>
       <c r="O9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P9">
         <v>1</v>
@@ -4688,13 +4684,13 @@
         <v>0</v>
       </c>
       <c r="W9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="X9" t="s">
         <v>99</v>
       </c>
       <c r="Y9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z9">
         <v>3</v>
@@ -4721,13 +4717,13 @@
         <v>44</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -4775,13 +4771,13 @@
         <v>0</v>
       </c>
       <c r="W10" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="X10" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="Y10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z10">
         <v>3</v>
@@ -4808,13 +4804,13 @@
         <v>45</v>
       </c>
       <c r="E11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -4862,13 +4858,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="X11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="Y11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="Z11">
         <v>6</v>
@@ -4898,10 +4894,10 @@
         <v>111</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -4949,10 +4945,10 @@
         <v>0</v>
       </c>
       <c r="W12" t="s">
+        <v>162</v>
+      </c>
+      <c r="X12" t="s">
         <v>163</v>
-      </c>
-      <c r="X12" t="s">
-        <v>164</v>
       </c>
       <c r="Y12" t="s">
         <v>101</v>
@@ -5008,7 +5004,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -5068,7 +5064,7 @@
         <v>98</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>19</v>
@@ -5095,10 +5091,10 @@
         <v>72</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -5122,7 +5118,7 @@
         <v>8</v>
       </c>
       <c r="O2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -5146,10 +5142,10 @@
         <v>0</v>
       </c>
       <c r="W2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="X2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y2" t="s">
         <v>101</v>
@@ -5176,16 +5172,16 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E3" t="s">
+        <v>166</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="G3" s="4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -5233,10 +5229,10 @@
         <v>0</v>
       </c>
       <c r="W3" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="X3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y3" t="s">
         <v>101</v>
@@ -5269,10 +5265,10 @@
         <v>77</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -5320,10 +5316,10 @@
         <v>0</v>
       </c>
       <c r="W4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y4" t="s">
         <v>101</v>
@@ -5356,10 +5352,10 @@
         <v>82</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -5407,13 +5403,13 @@
         <v>0</v>
       </c>
       <c r="W5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="X5" t="s">
         <v>99</v>
       </c>
       <c r="Y5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z5">
         <v>3</v>
@@ -5443,10 +5439,10 @@
         <v>64</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -5494,10 +5490,10 @@
         <v>0</v>
       </c>
       <c r="W6" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="X6" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="Y6" t="s">
         <v>101</v>
@@ -5533,7 +5529,7 @@
         <v>80</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -5581,10 +5577,10 @@
         <v>0</v>
       </c>
       <c r="W7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y7" t="s">
         <v>101</v>
@@ -5620,7 +5616,7 @@
         <v>88</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -5668,10 +5664,10 @@
         <v>0</v>
       </c>
       <c r="W8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="X8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="Y8" t="s">
         <v>101</v>
@@ -5704,10 +5700,10 @@
         <v>81</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -5755,13 +5751,13 @@
         <v>0</v>
       </c>
       <c r="W9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z9">
         <v>3</v>
@@ -5794,7 +5790,7 @@
         <v>79</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -5842,13 +5838,13 @@
         <v>0</v>
       </c>
       <c r="W10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="Z10">
         <v>3</v>
@@ -5878,10 +5874,10 @@
         <v>86</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -5929,10 +5925,10 @@
         <v>0</v>
       </c>
       <c r="W11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Y11" t="s">
         <v>101</v>
@@ -6016,7 +6012,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="X12" s="2" t="s">
         <v>102</v>
@@ -6055,7 +6051,7 @@
         <v>109</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>114</v>
+        <v>223</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -6103,10 +6099,10 @@
         <v>0</v>
       </c>
       <c r="W13" t="s">
+        <v>164</v>
+      </c>
+      <c r="X13" t="s">
         <v>165</v>
-      </c>
-      <c r="X13" t="s">
-        <v>166</v>
       </c>
       <c r="Y13" t="s">
         <v>101</v>
@@ -6160,7 +6156,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -6220,7 +6216,7 @@
         <v>98</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>19</v>
@@ -6250,7 +6246,7 @@
         <v>68</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H2" s="5">
         <v>0</v>
@@ -6298,10 +6294,10 @@
         <v>0</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y2" s="5" t="s">
         <v>101</v>
@@ -6334,10 +6330,10 @@
         <v>76</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H3" s="5">
         <v>0</v>
@@ -6385,10 +6381,10 @@
         <v>0</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y3" s="5" t="s">
         <v>101</v>
@@ -6421,10 +6417,10 @@
         <v>75</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H4" s="5">
         <v>0</v>
@@ -6472,10 +6468,10 @@
         <v>0</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y4" s="5" t="s">
         <v>101</v>
@@ -6508,10 +6504,10 @@
         <v>107</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H5" s="5">
         <v>0</v>
@@ -6559,10 +6555,10 @@
         <v>0</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X5" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y5" s="5" t="s">
         <v>101</v>
@@ -6592,13 +6588,13 @@
         <v>61</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H6" s="5">
         <v>0</v>
@@ -6646,10 +6642,10 @@
         <v>0</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y6" s="5" t="s">
         <v>101</v>
@@ -6682,10 +6678,10 @@
         <v>74</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H7" s="5">
         <v>0</v>
@@ -6733,10 +6729,10 @@
         <v>0</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X7" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y7" s="5" t="s">
         <v>101</v>
@@ -6769,10 +6765,10 @@
         <v>105</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H8" s="5">
         <v>0</v>
@@ -6820,10 +6816,10 @@
         <v>0</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y8" s="5" t="s">
         <v>101</v>
@@ -6856,7 +6852,7 @@
         <v>108</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>110</v>
@@ -6907,10 +6903,10 @@
         <v>0</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="X9" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y9" s="5" t="s">
         <v>100</v>

</xml_diff>